<commit_message>
Fix public_sector cfda_number type mismatch; strengthen reference-shift callout
QA caught a real bug: Grants.cfda_number was stored as a float (66.818)
while Programs.cfda_number was stored as text ("14.850") -- the required
XLOOKUP join between them would have returned #N/A on every row. Forced
both to matching string dtype when reading the source CSV. Also adds an
explicit copy/paste-shifts-references callout to CHECKLIST_TIMELINE.md
(previously only indirectly covered).
</commit_message>
<xml_diff>
--- a/starter/public_sector_workbook.xlsx
+++ b/starter/public_sector_workbook.xlsx
@@ -577,8 +577,10 @@
           <t>Environmental Protection Agency</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>66.818</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>66.818</t>
+        </is>
       </c>
       <c r="E2" t="n">
         <v>500000</v>
@@ -621,8 +623,10 @@
           <t>Environmental Protection Agency</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>66.818</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>66.818</t>
+        </is>
       </c>
       <c r="E3" t="n">
         <v>500000</v>
@@ -666,8 +670,10 @@
           <t>Environmental Protection Agency</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>66.818</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>66.818</t>
+        </is>
       </c>
       <c r="E4" t="n">
         <v>300000</v>
@@ -710,8 +716,10 @@
           <t>Environmental Protection Agency</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>66.818</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>66.818</t>
+        </is>
       </c>
       <c r="E5" t="n">
         <v>300000</v>
@@ -754,8 +762,10 @@
           <t>Environmental Protection Agency</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>66.818</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>66.818</t>
+        </is>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -798,8 +808,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>14.218</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E7" t="n">
         <v>1862177</v>
@@ -852,8 +864,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>14.218</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E8" t="n">
         <v>1804614</v>
@@ -906,8 +920,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>14.218</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E9" t="n">
         <v>1784484</v>
@@ -950,8 +966,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>14.218</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E10" t="n">
         <v>1718460</v>
@@ -1004,8 +1022,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>14.218</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E11" t="n">
         <v>1184874.54</v>
@@ -1044,8 +1064,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>14.218</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E12" t="n">
         <v>1025943</v>
@@ -1098,8 +1120,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>14.218</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E13" t="n">
         <v>933493</v>
@@ -1138,8 +1162,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>14.218</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E14" t="n">
         <v>658032</v>
@@ -1192,8 +1218,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>14.218</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E15" t="n">
         <v>350085</v>
@@ -1246,8 +1274,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>14.218</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E16" t="n">
         <v>325064</v>
@@ -1300,8 +1330,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>14.218</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E17" t="n">
         <v>204430</v>
@@ -1344,8 +1376,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>14.218</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E18" t="n">
         <v>189567</v>
@@ -1398,8 +1432,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>14.218</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>14.218</t>
+        </is>
       </c>
       <c r="E19" t="n">
         <v>172393</v>
@@ -1452,8 +1488,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>14.267</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E20" t="n">
         <v>829072</v>
@@ -1496,8 +1534,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>14.267</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E21" t="n">
         <v>720257</v>
@@ -1540,8 +1580,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>14.267</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E22" t="n">
         <v>715530</v>
@@ -1584,8 +1626,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>14.267</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E23" t="n">
         <v>593472.5699999999</v>
@@ -1628,8 +1672,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>14.267</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E24" t="n">
         <v>455038.64</v>
@@ -1672,8 +1718,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>14.267</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E25" t="n">
         <v>389625</v>
@@ -1716,8 +1764,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>14.267</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E26" t="n">
         <v>365075</v>
@@ -1760,8 +1810,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>14.267</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E27" t="n">
         <v>354559.64</v>
@@ -1804,8 +1856,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>14.267</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E28" t="n">
         <v>345134</v>
@@ -1848,8 +1902,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>14.267</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E29" t="n">
         <v>291324</v>
@@ -1892,8 +1948,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>14.267</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E30" t="n">
         <v>241180</v>
@@ -1936,8 +1994,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>14.267</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E31" t="n">
         <v>221280.5</v>
@@ -1980,8 +2040,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>14.267</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E32" t="n">
         <v>217465.15</v>
@@ -2024,8 +2086,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>14.267</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E33" t="n">
         <v>214814</v>
@@ -2068,8 +2132,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>14.267</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E34" t="n">
         <v>211309</v>
@@ -2112,8 +2178,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>14.267</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E35" t="n">
         <v>204982.55</v>
@@ -2156,8 +2224,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>14.267</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E36" t="n">
         <v>194069</v>
@@ -2200,8 +2270,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>14.267</v>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E37" t="n">
         <v>180544</v>
@@ -2244,8 +2316,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>14.267</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E38" t="n">
         <v>173667</v>
@@ -2288,8 +2362,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>14.267</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E39" t="n">
         <v>168870</v>
@@ -2332,8 +2408,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>14.267</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E40" t="n">
         <v>166347</v>
@@ -2376,8 +2454,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>14.267</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E41" t="n">
         <v>163215</v>
@@ -2420,8 +2500,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>14.267</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E42" t="n">
         <v>144717</v>
@@ -2464,8 +2546,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>14.267</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E43" t="n">
         <v>135156.89</v>
@@ -2508,8 +2592,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>14.267</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E44" t="n">
         <v>133934.7</v>
@@ -2552,8 +2638,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>14.267</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E45" t="n">
         <v>128767</v>
@@ -2596,8 +2684,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>14.267</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E46" t="n">
         <v>119181</v>
@@ -2640,8 +2730,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>14.267</v>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E47" t="n">
         <v>118264</v>
@@ -2684,8 +2776,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>14.267</v>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E48" t="n">
         <v>101596</v>
@@ -2728,8 +2822,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>14.267</v>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E49" t="n">
         <v>99894.12</v>
@@ -2772,8 +2868,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>14.267</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E50" t="n">
         <v>99655.81</v>
@@ -2816,8 +2914,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>14.267</v>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E51" t="n">
         <v>90792</v>
@@ -2860,8 +2960,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>14.267</v>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E52" t="n">
         <v>89452</v>
@@ -2904,8 +3006,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>14.267</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E53" t="n">
         <v>88924</v>
@@ -2948,8 +3052,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>14.267</v>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E54" t="n">
         <v>82827</v>
@@ -2992,8 +3098,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>14.267</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E55" t="n">
         <v>82156</v>
@@ -3036,8 +3144,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>14.267</v>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E56" t="n">
         <v>72959.8</v>
@@ -3080,8 +3190,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>14.267</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E57" t="n">
         <v>63913.87</v>
@@ -3124,8 +3236,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>14.267</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>14.267</t>
+        </is>
       </c>
       <c r="E58" t="n">
         <v>31716</v>
@@ -3168,8 +3282,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>14.251</v>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>14.251</t>
+        </is>
       </c>
       <c r="E59" t="n">
         <v>4116279</v>
@@ -3213,8 +3329,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D60" t="n">
-        <v>14.251</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>14.251</t>
+        </is>
       </c>
       <c r="E60" t="n">
         <v>4000000</v>
@@ -3257,8 +3375,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>14.251</v>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>14.251</t>
+        </is>
       </c>
       <c r="E61" t="n">
         <v>3000000</v>
@@ -3301,8 +3421,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>14.251</v>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>14.251</t>
+        </is>
       </c>
       <c r="E62" t="n">
         <v>2000000</v>
@@ -3346,8 +3468,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D63" t="n">
-        <v>14.251</v>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>14.251</t>
+        </is>
       </c>
       <c r="E63" t="n">
         <v>1500000</v>
@@ -3390,8 +3514,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D64" t="n">
-        <v>14.251</v>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>14.251</t>
+        </is>
       </c>
       <c r="E64" t="n">
         <v>500000</v>
@@ -3434,8 +3560,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D65" t="n">
-        <v>14.231</v>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>14.231</t>
+        </is>
       </c>
       <c r="E65" t="n">
         <v>2493328</v>
@@ -3478,8 +3606,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D66" t="n">
-        <v>14.231</v>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>14.231</t>
+        </is>
       </c>
       <c r="E66" t="n">
         <v>159511</v>
@@ -3522,8 +3652,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D67" t="n">
-        <v>14.231</v>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>14.231</t>
+        </is>
       </c>
       <c r="E67" t="n">
         <v>151468</v>
@@ -3566,8 +3698,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D68" t="n">
-        <v>14.231</v>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>14.231</t>
+        </is>
       </c>
       <c r="E68" t="n">
         <v>148882</v>
@@ -3610,8 +3744,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D69" t="n">
-        <v>14.896</v>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>14.896</t>
+        </is>
       </c>
       <c r="E69" t="n">
         <v>140000</v>
@@ -3654,8 +3790,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D70" t="n">
-        <v>14.896</v>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>14.896</t>
+        </is>
       </c>
       <c r="E70" t="n">
         <v>109352</v>
@@ -3698,8 +3836,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D71" t="n">
-        <v>14.896</v>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>14.896</t>
+        </is>
       </c>
       <c r="E71" t="n">
         <v>74438</v>
@@ -3742,8 +3882,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D72" t="n">
-        <v>14.896</v>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>14.896</t>
+        </is>
       </c>
       <c r="E72" t="n">
         <v>59006.84</v>
@@ -3786,8 +3928,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D73" t="n">
-        <v>14.896</v>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>14.896</t>
+        </is>
       </c>
       <c r="E73" t="n">
         <v>55000</v>
@@ -3830,8 +3974,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D74" t="n">
-        <v>14.239</v>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E74" t="n">
         <v>7489050</v>
@@ -3876,8 +4022,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D75" t="n">
-        <v>14.239</v>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E75" t="n">
         <v>1199888</v>
@@ -3920,8 +4068,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D76" t="n">
-        <v>14.239</v>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E76" t="n">
         <v>884706</v>
@@ -3964,8 +4114,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D77" t="n">
-        <v>14.239</v>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E77" t="n">
         <v>877289</v>
@@ -4010,8 +4162,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D78" t="n">
-        <v>14.239</v>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E78" t="n">
         <v>868030</v>
@@ -4054,8 +4208,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D79" t="n">
-        <v>14.239</v>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E79" t="n">
         <v>744108</v>
@@ -4098,8 +4254,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D80" t="n">
-        <v>14.239</v>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E80" t="n">
         <v>710287.23</v>
@@ -4144,8 +4302,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D81" t="n">
-        <v>14.239</v>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E81" t="n">
         <v>675768.3</v>
@@ -4190,8 +4350,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D82" t="n">
-        <v>14.239</v>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E82" t="n">
         <v>571221</v>
@@ -4236,8 +4398,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D83" t="n">
-        <v>14.239</v>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E83" t="n">
         <v>552117</v>
@@ -4282,8 +4446,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D84" t="n">
-        <v>14.239</v>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E84" t="n">
         <v>463432</v>
@@ -4322,8 +4488,10 @@
           <t>Assistant Secretary for Community Planning and Development</t>
         </is>
       </c>
-      <c r="D85" t="n">
-        <v>14.239</v>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>14.239</t>
+        </is>
       </c>
       <c r="E85" t="n">
         <v>299732.18</v>
@@ -4368,8 +4536,10 @@
           <t>Assistant Secretary for Housing--Federal Housing Commissioner</t>
         </is>
       </c>
-      <c r="D86" t="n">
-        <v>14.191</v>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>14.191</t>
+        </is>
       </c>
       <c r="E86" t="n">
         <v>150961.78</v>
@@ -4412,8 +4582,10 @@
           <t>Assistant Secretary for Housing--Federal Housing Commissioner</t>
         </is>
       </c>
-      <c r="D87" t="n">
-        <v>14.191</v>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>14.191</t>
+        </is>
       </c>
       <c r="E87" t="n">
         <v>6756.14</v>
@@ -4456,8 +4628,10 @@
           <t>Assistant Secretary for Housing--Federal Housing Commissioner</t>
         </is>
       </c>
-      <c r="D88" t="n">
-        <v>14.191</v>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>14.191</t>
+        </is>
       </c>
       <c r="E88" t="n">
         <v>5392.96</v>
@@ -4500,8 +4674,10 @@
           <t>Assistant Secretary for Housing--Federal Housing Commissioner</t>
         </is>
       </c>
-      <c r="D89" t="n">
-        <v>14.191</v>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>14.191</t>
+        </is>
       </c>
       <c r="E89" t="n">
         <v>0</v>
@@ -4540,8 +4716,10 @@
           <t>Assistant Secretary for Housing--Federal Housing Commissioner</t>
         </is>
       </c>
-      <c r="D90" t="n">
-        <v>14.191</v>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>14.191</t>
+        </is>
       </c>
       <c r="E90" t="n">
         <v>0</v>
@@ -4580,8 +4758,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D91" t="n">
-        <v>14.872</v>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E91" t="n">
         <v>6501354</v>
@@ -4624,8 +4804,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D92" t="n">
-        <v>14.872</v>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E92" t="n">
         <v>4701254</v>
@@ -4679,8 +4861,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D93" t="n">
-        <v>14.872</v>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E93" t="n">
         <v>3707622</v>
@@ -4723,8 +4907,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D94" t="n">
-        <v>14.872</v>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E94" t="n">
         <v>2854223</v>
@@ -4778,8 +4964,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D95" t="n">
-        <v>14.872</v>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E95" t="n">
         <v>2850280</v>
@@ -4822,8 +5010,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D96" t="n">
-        <v>14.872</v>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E96" t="n">
         <v>2717487</v>
@@ -4866,8 +5056,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D97" t="n">
-        <v>14.872</v>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E97" t="n">
         <v>1311688</v>
@@ -4921,8 +5113,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D98" t="n">
-        <v>14.872</v>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E98" t="n">
         <v>1292357</v>
@@ -4965,8 +5159,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>14.872</v>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E99" t="n">
         <v>1204446</v>
@@ -5020,8 +5216,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D100" t="n">
-        <v>14.872</v>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E100" t="n">
         <v>974527</v>
@@ -5075,8 +5273,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D101" t="n">
-        <v>14.872</v>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E101" t="n">
         <v>927183</v>
@@ -5119,8 +5319,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D102" t="n">
-        <v>14.872</v>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E102" t="n">
         <v>870058</v>
@@ -5174,8 +5376,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D103" t="n">
-        <v>14.872</v>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E103" t="n">
         <v>863463</v>
@@ -5218,8 +5422,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D104" t="n">
-        <v>14.872</v>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E104" t="n">
         <v>796105</v>
@@ -5262,8 +5468,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D105" t="n">
-        <v>14.872</v>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E105" t="n">
         <v>754424</v>
@@ -5317,8 +5525,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D106" t="n">
-        <v>14.872</v>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E106" t="n">
         <v>704163</v>
@@ -5361,8 +5571,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D107" t="n">
-        <v>14.872</v>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E107" t="n">
         <v>674852</v>
@@ -5405,8 +5617,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D108" t="n">
-        <v>14.872</v>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E108" t="n">
         <v>658500</v>
@@ -5460,8 +5674,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D109" t="n">
-        <v>14.872</v>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E109" t="n">
         <v>599700</v>
@@ -5504,8 +5720,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D110" t="n">
-        <v>14.872</v>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E110" t="n">
         <v>550786</v>
@@ -5559,8 +5777,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D111" t="n">
-        <v>14.872</v>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E111" t="n">
         <v>479895</v>
@@ -5603,8 +5823,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D112" t="n">
-        <v>14.872</v>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E112" t="n">
         <v>423672</v>
@@ -5647,8 +5869,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D113" t="n">
-        <v>14.872</v>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E113" t="n">
         <v>393148</v>
@@ -5691,8 +5915,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D114" t="n">
-        <v>14.872</v>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E114" t="n">
         <v>362889</v>
@@ -5735,8 +5961,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D115" t="n">
-        <v>14.872</v>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E115" t="n">
         <v>354291</v>
@@ -5779,8 +6007,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D116" t="n">
-        <v>14.872</v>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E116" t="n">
         <v>330348</v>
@@ -5834,8 +6064,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D117" t="n">
-        <v>14.872</v>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E117" t="n">
         <v>322030</v>
@@ -5878,8 +6110,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D118" t="n">
-        <v>14.872</v>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E118" t="n">
         <v>293607</v>
@@ -5922,8 +6156,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D119" t="n">
-        <v>14.872</v>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E119" t="n">
         <v>271991</v>
@@ -5966,8 +6202,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D120" t="n">
-        <v>14.872</v>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E120" t="n">
         <v>271353</v>
@@ -6010,8 +6248,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D121" t="n">
-        <v>14.872</v>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E121" t="n">
         <v>267157</v>
@@ -6054,8 +6294,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D122" t="n">
-        <v>14.872</v>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>14.872</t>
+        </is>
       </c>
       <c r="E122" t="n">
         <v>140261</v>
@@ -6098,8 +6340,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D123" t="n">
-        <v>14.85</v>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E123" t="n">
         <v>3150764</v>
@@ -6142,8 +6386,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D124" t="n">
-        <v>14.85</v>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E124" t="n">
         <v>2759361</v>
@@ -6186,8 +6432,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D125" t="n">
-        <v>14.85</v>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E125" t="n">
         <v>2670204</v>
@@ -6230,8 +6478,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D126" t="n">
-        <v>14.85</v>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E126" t="n">
         <v>2439599</v>
@@ -6274,8 +6524,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D127" t="n">
-        <v>14.85</v>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E127" t="n">
         <v>2340001</v>
@@ -6318,8 +6570,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D128" t="n">
-        <v>14.85</v>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E128" t="n">
         <v>2176058</v>
@@ -6362,8 +6616,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D129" t="n">
-        <v>14.85</v>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E129" t="n">
         <v>2139166</v>
@@ -6406,8 +6662,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D130" t="n">
-        <v>14.85</v>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E130" t="n">
         <v>1313705</v>
@@ -6450,8 +6708,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D131" t="n">
-        <v>14.85</v>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E131" t="n">
         <v>1280445</v>
@@ -6494,8 +6754,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D132" t="n">
-        <v>14.85</v>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E132" t="n">
         <v>1220799</v>
@@ -6538,8 +6800,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D133" t="n">
-        <v>14.85</v>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E133" t="n">
         <v>1162444</v>
@@ -6582,8 +6846,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D134" t="n">
-        <v>14.85</v>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E134" t="n">
         <v>1148168</v>
@@ -6626,8 +6892,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D135" t="n">
-        <v>14.85</v>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E135" t="n">
         <v>978172</v>
@@ -6670,8 +6938,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D136" t="n">
-        <v>14.85</v>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E136" t="n">
         <v>927278</v>
@@ -6714,8 +6984,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D137" t="n">
-        <v>14.85</v>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E137" t="n">
         <v>797212</v>
@@ -6758,8 +7030,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D138" t="n">
-        <v>14.85</v>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E138" t="n">
         <v>747232</v>
@@ -6802,8 +7076,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D139" t="n">
-        <v>14.85</v>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E139" t="n">
         <v>710426</v>
@@ -6846,8 +7122,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D140" t="n">
-        <v>14.85</v>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E140" t="n">
         <v>693174</v>
@@ -6890,8 +7168,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D141" t="n">
-        <v>14.85</v>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E141" t="n">
         <v>686217</v>
@@ -6934,8 +7214,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D142" t="n">
-        <v>14.85</v>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E142" t="n">
         <v>681597</v>
@@ -6978,8 +7260,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D143" t="n">
-        <v>14.85</v>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E143" t="n">
         <v>672644</v>
@@ -7022,8 +7306,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D144" t="n">
-        <v>14.85</v>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E144" t="n">
         <v>662149</v>
@@ -7066,8 +7352,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D145" t="n">
-        <v>14.85</v>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E145" t="n">
         <v>661950</v>
@@ -7110,8 +7398,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D146" t="n">
-        <v>14.85</v>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E146" t="n">
         <v>657775</v>
@@ -7154,8 +7444,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D147" t="n">
-        <v>14.85</v>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E147" t="n">
         <v>644261</v>
@@ -7198,8 +7490,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D148" t="n">
-        <v>14.85</v>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E148" t="n">
         <v>630388</v>
@@ -7242,8 +7536,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D149" t="n">
-        <v>14.85</v>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E149" t="n">
         <v>622314</v>
@@ -7286,8 +7582,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D150" t="n">
-        <v>14.85</v>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E150" t="n">
         <v>620676</v>
@@ -7330,8 +7628,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D151" t="n">
-        <v>14.85</v>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E151" t="n">
         <v>620138</v>
@@ -7374,8 +7674,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D152" t="n">
-        <v>14.85</v>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E152" t="n">
         <v>612495</v>
@@ -7418,8 +7720,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D153" t="n">
-        <v>14.85</v>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E153" t="n">
         <v>611637</v>
@@ -7462,8 +7766,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D154" t="n">
-        <v>14.85</v>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E154" t="n">
         <v>607291</v>
@@ -7506,8 +7812,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D155" t="n">
-        <v>14.85</v>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E155" t="n">
         <v>607194</v>
@@ -7550,8 +7858,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D156" t="n">
-        <v>14.85</v>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E156" t="n">
         <v>600537</v>
@@ -7594,8 +7904,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D157" t="n">
-        <v>14.85</v>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E157" t="n">
         <v>594915</v>
@@ -7638,8 +7950,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D158" t="n">
-        <v>14.85</v>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E158" t="n">
         <v>593151</v>
@@ -7682,8 +7996,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D159" t="n">
-        <v>14.85</v>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E159" t="n">
         <v>581768</v>
@@ -7726,8 +8042,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D160" t="n">
-        <v>14.85</v>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E160" t="n">
         <v>581233</v>
@@ -7770,8 +8088,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D161" t="n">
-        <v>14.85</v>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E161" t="n">
         <v>580488</v>
@@ -7814,8 +8134,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D162" t="n">
-        <v>14.85</v>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E162" t="n">
         <v>575582</v>
@@ -7858,8 +8180,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D163" t="n">
-        <v>14.85</v>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E163" t="n">
         <v>556204</v>
@@ -7902,8 +8226,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D164" t="n">
-        <v>14.85</v>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E164" t="n">
         <v>548985</v>
@@ -7946,8 +8272,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D165" t="n">
-        <v>14.85</v>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E165" t="n">
         <v>536348</v>
@@ -7990,8 +8318,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D166" t="n">
-        <v>14.85</v>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E166" t="n">
         <v>532927</v>
@@ -8034,8 +8364,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D167" t="n">
-        <v>14.85</v>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E167" t="n">
         <v>530540</v>
@@ -8078,8 +8410,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D168" t="n">
-        <v>14.85</v>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E168" t="n">
         <v>521727</v>
@@ -8122,8 +8456,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D169" t="n">
-        <v>14.85</v>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E169" t="n">
         <v>516822</v>
@@ -8166,8 +8502,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D170" t="n">
-        <v>14.85</v>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E170" t="n">
         <v>513252</v>
@@ -8210,8 +8548,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D171" t="n">
-        <v>14.85</v>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E171" t="n">
         <v>509284</v>
@@ -8254,8 +8594,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D172" t="n">
-        <v>14.85</v>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E172" t="n">
         <v>495896</v>
@@ -8298,8 +8640,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D173" t="n">
-        <v>14.85</v>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E173" t="n">
         <v>492754</v>
@@ -8342,8 +8686,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D174" t="n">
-        <v>14.85</v>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E174" t="n">
         <v>489005</v>
@@ -8386,8 +8732,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D175" t="n">
-        <v>14.85</v>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E175" t="n">
         <v>466912</v>
@@ -8430,8 +8778,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D176" t="n">
-        <v>14.85</v>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E176" t="n">
         <v>435992</v>
@@ -8474,8 +8824,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D177" t="n">
-        <v>14.85</v>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E177" t="n">
         <v>429965</v>
@@ -8518,8 +8870,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D178" t="n">
-        <v>14.85</v>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E178" t="n">
         <v>416934</v>
@@ -8562,8 +8916,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D179" t="n">
-        <v>14.85</v>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E179" t="n">
         <v>410397</v>
@@ -8606,8 +8962,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D180" t="n">
-        <v>14.85</v>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E180" t="n">
         <v>408819</v>
@@ -8650,8 +9008,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D181" t="n">
-        <v>14.85</v>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E181" t="n">
         <v>398287</v>
@@ -8694,8 +9054,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D182" t="n">
-        <v>14.85</v>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E182" t="n">
         <v>397656</v>
@@ -8738,8 +9100,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D183" t="n">
-        <v>14.85</v>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E183" t="n">
         <v>389668</v>
@@ -8782,8 +9146,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D184" t="n">
-        <v>14.85</v>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E184" t="n">
         <v>378698</v>
@@ -8826,8 +9192,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D185" t="n">
-        <v>14.85</v>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E185" t="n">
         <v>367847</v>
@@ -8870,8 +9238,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D186" t="n">
-        <v>14.85</v>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E186" t="n">
         <v>365560</v>
@@ -8914,8 +9284,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D187" t="n">
-        <v>14.85</v>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E187" t="n">
         <v>349994</v>
@@ -8958,8 +9330,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D188" t="n">
-        <v>14.85</v>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E188" t="n">
         <v>347042</v>
@@ -9002,8 +9376,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D189" t="n">
-        <v>14.85</v>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E189" t="n">
         <v>346478</v>
@@ -9046,8 +9422,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D190" t="n">
-        <v>14.85</v>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E190" t="n">
         <v>331113</v>
@@ -9090,8 +9468,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D191" t="n">
-        <v>14.85</v>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E191" t="n">
         <v>325981</v>
@@ -9134,8 +9514,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D192" t="n">
-        <v>14.85</v>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E192" t="n">
         <v>320474</v>
@@ -9178,8 +9560,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D193" t="n">
-        <v>14.85</v>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E193" t="n">
         <v>300797</v>
@@ -9222,8 +9606,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>14.85</v>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E194" t="n">
         <v>299802</v>
@@ -9266,8 +9652,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D195" t="n">
-        <v>14.85</v>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E195" t="n">
         <v>292394</v>
@@ -9310,8 +9698,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D196" t="n">
-        <v>14.85</v>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E196" t="n">
         <v>279608</v>
@@ -9354,8 +9744,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D197" t="n">
-        <v>14.85</v>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E197" t="n">
         <v>273078</v>
@@ -9398,8 +9790,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D198" t="n">
-        <v>14.85</v>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E198" t="n">
         <v>260882</v>
@@ -9442,8 +9836,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D199" t="n">
-        <v>14.85</v>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E199" t="n">
         <v>256228</v>
@@ -9486,8 +9882,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D200" t="n">
-        <v>14.85</v>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E200" t="n">
         <v>247880</v>
@@ -9530,8 +9928,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D201" t="n">
-        <v>14.85</v>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E201" t="n">
         <v>244269</v>
@@ -9574,8 +9974,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D202" t="n">
-        <v>14.85</v>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E202" t="n">
         <v>240972</v>
@@ -9618,8 +10020,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D203" t="n">
-        <v>14.85</v>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E203" t="n">
         <v>237219</v>
@@ -9662,8 +10066,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D204" t="n">
-        <v>14.85</v>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E204" t="n">
         <v>234478</v>
@@ -9706,8 +10112,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D205" t="n">
-        <v>14.85</v>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E205" t="n">
         <v>225464</v>
@@ -9750,8 +10158,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D206" t="n">
-        <v>14.85</v>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E206" t="n">
         <v>222411</v>
@@ -9794,8 +10204,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D207" t="n">
-        <v>14.85</v>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E207" t="n">
         <v>218938</v>
@@ -9838,8 +10250,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D208" t="n">
-        <v>14.85</v>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E208" t="n">
         <v>218887</v>
@@ -9882,8 +10296,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D209" t="n">
-        <v>14.85</v>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E209" t="n">
         <v>212385</v>
@@ -9926,8 +10342,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D210" t="n">
-        <v>14.85</v>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E210" t="n">
         <v>200305</v>
@@ -9970,8 +10388,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D211" t="n">
-        <v>14.85</v>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E211" t="n">
         <v>198409</v>
@@ -10014,8 +10434,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D212" t="n">
-        <v>14.85</v>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E212" t="n">
         <v>195022</v>
@@ -10058,8 +10480,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D213" t="n">
-        <v>14.85</v>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E213" t="n">
         <v>193748</v>
@@ -10102,8 +10526,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D214" t="n">
-        <v>14.85</v>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E214" t="n">
         <v>173870</v>
@@ -10146,8 +10572,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D215" t="n">
-        <v>14.85</v>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E215" t="n">
         <v>165847</v>
@@ -10190,8 +10618,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D216" t="n">
-        <v>14.85</v>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E216" t="n">
         <v>154883</v>
@@ -10234,8 +10664,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D217" t="n">
-        <v>14.85</v>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E217" t="n">
         <v>150172</v>
@@ -10278,8 +10710,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D218" t="n">
-        <v>14.85</v>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E218" t="n">
         <v>136548</v>
@@ -10322,8 +10756,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D219" t="n">
-        <v>14.85</v>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E219" t="n">
         <v>129638</v>
@@ -10366,8 +10802,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D220" t="n">
-        <v>14.85</v>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E220" t="n">
         <v>128582</v>
@@ -10410,8 +10848,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D221" t="n">
-        <v>14.85</v>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E221" t="n">
         <v>112044</v>
@@ -10454,8 +10894,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D222" t="n">
-        <v>14.85</v>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E222" t="n">
         <v>100780</v>
@@ -10498,8 +10940,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D223" t="n">
-        <v>14.85</v>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E223" t="n">
         <v>99536</v>
@@ -10542,8 +10986,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D224" t="n">
-        <v>14.85</v>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E224" t="n">
         <v>97074</v>
@@ -10586,8 +11032,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D225" t="n">
-        <v>14.85</v>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E225" t="n">
         <v>97014</v>
@@ -10630,8 +11078,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D226" t="n">
-        <v>14.85</v>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E226" t="n">
         <v>92516</v>
@@ -10674,8 +11124,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D227" t="n">
-        <v>14.85</v>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E227" t="n">
         <v>90750</v>
@@ -10718,8 +11170,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D228" t="n">
-        <v>14.85</v>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E228" t="n">
         <v>86716</v>
@@ -10762,8 +11216,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D229" t="n">
-        <v>14.85</v>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E229" t="n">
         <v>86257</v>
@@ -10806,8 +11262,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D230" t="n">
-        <v>14.85</v>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E230" t="n">
         <v>85638</v>
@@ -10850,8 +11308,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D231" t="n">
-        <v>14.85</v>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E231" t="n">
         <v>82840</v>
@@ -10894,8 +11354,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D232" t="n">
-        <v>14.85</v>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E232" t="n">
         <v>82704</v>
@@ -10938,8 +11400,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D233" t="n">
-        <v>14.85</v>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E233" t="n">
         <v>80343</v>
@@ -10982,8 +11446,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D234" t="n">
-        <v>14.85</v>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E234" t="n">
         <v>78305</v>
@@ -11026,8 +11492,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D235" t="n">
-        <v>14.85</v>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E235" t="n">
         <v>53913</v>
@@ -11070,8 +11538,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D236" t="n">
-        <v>14.85</v>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E236" t="n">
         <v>23029</v>
@@ -11114,8 +11584,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D237" t="n">
-        <v>14.85</v>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E237" t="n">
         <v>22770</v>
@@ -11158,8 +11630,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D238" t="n">
-        <v>14.85</v>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E238" t="n">
         <v>16300</v>
@@ -11202,8 +11676,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D239" t="n">
-        <v>14.85</v>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E239" t="n">
         <v>8549</v>
@@ -11246,8 +11722,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D240" t="n">
-        <v>14.85</v>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E240" t="n">
         <v>5634</v>
@@ -11290,8 +11768,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D241" t="n">
-        <v>14.85</v>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E241" t="n">
         <v>5125</v>
@@ -11334,8 +11814,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D242" t="n">
-        <v>14.85</v>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E242" t="n">
         <v>3898</v>
@@ -11378,8 +11860,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D243" t="n">
-        <v>14.85</v>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E243" t="n">
         <v>3757</v>
@@ -11422,8 +11906,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D244" t="n">
-        <v>14.85</v>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E244" t="n">
         <v>3537</v>
@@ -11466,8 +11952,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D245" t="n">
-        <v>14.85</v>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E245" t="n">
         <v>3224</v>
@@ -11510,8 +11998,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D246" t="n">
-        <v>14.85</v>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E246" t="n">
         <v>3222</v>
@@ -11554,8 +12044,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D247" t="n">
-        <v>14.85</v>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E247" t="n">
         <v>3121</v>
@@ -11598,8 +12090,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D248" t="n">
-        <v>14.85</v>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E248" t="n">
         <v>1595</v>
@@ -11642,8 +12136,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D249" t="n">
-        <v>14.85</v>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E249" t="n">
         <v>0</v>
@@ -11682,8 +12178,10 @@
           <t>Assistant Secretary for Public and Indian Housing</t>
         </is>
       </c>
-      <c r="D250" t="n">
-        <v>14.85</v>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>14.850</t>
+        </is>
       </c>
       <c r="E250" t="n">
         <v>0</v>

</xml_diff>